<commit_message>
Correção Readme e documentação
</commit_message>
<xml_diff>
--- a/documentacao_planejamento_testes/relatorios/relatorio_bugs_api_sicredi.xlsx
+++ b/documentacao_planejamento_testes/relatorios/relatorio_bugs_api_sicredi.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo Executivo" sheetId="1" r:id="R7280eff87b7145a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relatório de Bugs" sheetId="2" r:id="Rd8940a3fa6ec46e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critérios e Métricas" sheetId="3" r:id="Rb29e8469deed46ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo Executivo" sheetId="1" r:id="R1942b4c4ba0f4d4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relatório de Bugs" sheetId="2" r:id="Rdc1e22b7c9584687"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critérios e Métricas" sheetId="3" r:id="R338b302ccc804c18"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -61,7 +61,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -91,6 +91,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="F8FAFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="1F4E78"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -190,7 +200,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="52">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -302,6 +312,27 @@
     <x:xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -314,7 +345,7 @@
         <x:color rgb="991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -325,7 +356,7 @@
         <x:color rgb="92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -336,7 +367,7 @@
         <x:color rgb="166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="DCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -625,7 +656,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9a704684a392493e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc51ee66ebbd248ee"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -660,7 +691,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3a1a9d6a251e4131"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0da1ad2da57d462a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -670,8 +701,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaRelatorioBugs" displayName="TabelaRelatorioBugs" ref="A1:O30" headerRowCount="1">
-  <x:tableColumns count="15">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaRelatorioBugs" displayName="TabelaRelatorioBugs" ref="A1:L30" headerRowCount="1">
+  <x:tableColumns count="12">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Ref."/>
     <x:tableColumn id="3" name="Tipo"/>
@@ -684,9 +715,6 @@
     <x:tableColumn id="10" name="Comportamento observado"/>
     <x:tableColumn id="11" name="Resultado esperado"/>
     <x:tableColumn id="12" name="Impacto"/>
-    <x:tableColumn id="13" name="Evidência"/>
-    <x:tableColumn id="14" name="Labels"/>
-    <x:tableColumn id="15" name="Criado em"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -856,10 +884,8 @@
         <x:v>Relatório de Defeitos e Melhorias - API Sicredi</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Resumo executivo gerado a partir do backlog de bugs do projeto. Extração: 18/05/2026.</x:v>
-      </x:c>
+    <x:row r="2" ht="4.5" customHeight="1">
+      <x:c r="A2" s="7"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="str">
@@ -1110,7 +1136,7 @@
     <x:mergeCell ref="A23:H23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf73fa1599b4829"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5615636b71d494a"/>
 </x:worksheet>
 </file>
 
@@ -1118,1432 +1144,1252 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10.09000015258789" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="7.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14.800000190734863" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="10.770000457763672" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="10.09000015258789" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="9.420000076293945" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13.460000038146973" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="15.479999542236328" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="41.720001220703125" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42.400001525878906" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="58.54999923706055" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="45.7599983215332" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="42.400001525878906" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="50.470001220703125" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="47.779998779296875" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="28.940000534057617" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="24.899999618530273" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="12.789999961853027" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="25.5" customHeight="1">
-      <x:c r="A1" s="49" t="str">
+    <x:row r="1" ht="22.5" customHeight="1">
+      <x:c r="A1" s="58" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B1" s="49" t="str">
+      <x:c r="B1" s="58" t="str">
         <x:v>Ref.</x:v>
       </x:c>
-      <x:c r="C1" s="49" t="str">
+      <x:c r="C1" s="58" t="str">
         <x:v>Tipo</x:v>
       </x:c>
-      <x:c r="D1" s="49" t="str">
+      <x:c r="D1" s="58" t="str">
         <x:v>Severidade</x:v>
       </x:c>
-      <x:c r="E1" s="49" t="str">
+      <x:c r="E1" s="58" t="str">
         <x:v>Prioridade</x:v>
       </x:c>
-      <x:c r="F1" s="49" t="str">
+      <x:c r="F1" s="58" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G1" s="49" t="str">
+      <x:c r="G1" s="58" t="str">
         <x:v>Método</x:v>
       </x:c>
-      <x:c r="H1" s="49" t="str">
+      <x:c r="H1" s="58" t="str">
         <x:v>Módulo</x:v>
       </x:c>
-      <x:c r="I1" s="49" t="str">
+      <x:c r="I1" s="58" t="str">
         <x:v>Título</x:v>
       </x:c>
-      <x:c r="J1" s="49" t="str">
+      <x:c r="J1" s="58" t="str">
         <x:v>Comportamento observado</x:v>
       </x:c>
-      <x:c r="K1" s="49" t="str">
+      <x:c r="K1" s="58" t="str">
         <x:v>Resultado esperado</x:v>
       </x:c>
-      <x:c r="L1" s="49" t="str">
+      <x:c r="L1" s="58" t="str">
         <x:v>Impacto</x:v>
       </x:c>
-      <x:c r="M1" s="49" t="str">
-        <x:v>Evidência</x:v>
-      </x:c>
-      <x:c r="N1" s="49" t="str">
-        <x:v>Labels</x:v>
-      </x:c>
-      <x:c r="O1" s="49" t="str">
-        <x:v>Criado em</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="64.5" customHeight="1">
-      <x:c r="A2" s="40" t="str">
+      <x:c r="M1"/>
+      <x:c r="N1"/>
+      <x:c r="O1"/>
+    </x:row>
+    <x:row r="2" ht="84" customHeight="1">
+      <x:c r="A2" s="52" t="str">
         <x:v>BUG-001</x:v>
       </x:c>
-      <x:c r="B2" s="41" t="str">
+      <x:c r="B2" s="52" t="str">
         <x:v>#1</x:v>
       </x:c>
-      <x:c r="C2" s="41" t="str">
+      <x:c r="C2" s="52" t="str">
         <x:v>Melhoria</x:v>
       </x:c>
-      <x:c r="D2" s="41" t="str">
+      <x:c r="D2" s="52" t="str">
         <x:v>Baixa</x:v>
       </x:c>
-      <x:c r="E2" s="41" t="str">
+      <x:c r="E2" s="52" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="F2" s="41" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G2" s="41" t="str">
+      <x:c r="F2" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G2" s="52" t="str">
         <x:v>GET</x:v>
       </x:c>
-      <x:c r="H2" s="41" t="str">
+      <x:c r="H2" s="52" t="str">
         <x:v>Restrições</x:v>
       </x:c>
-      <x:c r="I2" s="41" t="str">
+      <x:c r="I2" s="52" t="str">
         <x:v>Proibir busca de CPF com menos de 11 dígitos</x:v>
       </x:c>
-      <x:c r="J2" s="41" t="str">
+      <x:c r="J2" s="52" t="str">
         <x:v>Ao tentar utilizar a função de procurar CPF com restrições, a API aceita qualquer tamanho de CPF como instrução, para economizar tempo e recursos, o ideal seria que ele apenas aceitasse requisições de CPFs apenas com 11 dígitos.</x:v>
       </x:c>
-      <x:c r="K2" s="41" t="str">
+      <x:c r="K2" s="52" t="str">
         <x:v>Rejeitar CPF com menos de 11 dígitos e retornar validação clara.</x:v>
       </x:c>
-      <x:c r="L2" s="41" t="str">
+      <x:c r="L2" s="52" t="str">
         <x:v>Reduz precisão das validações e da comunicação da API para cenários de consulta.</x:v>
       </x:c>
-      <x:c r="M2" s="41" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N2" s="41" t="str">
-        <x:v>GET, Melhoria, Restrições</x:v>
-      </x:c>
-      <x:c r="O2" s="42" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="64.5" customHeight="1">
-      <x:c r="A3" s="43" t="str">
+      <x:c r="M2"/>
+      <x:c r="N2"/>
+      <x:c r="O2"/>
+    </x:row>
+    <x:row r="3" ht="84" customHeight="1">
+      <x:c r="A3" s="52" t="str">
         <x:v>BUG-002</x:v>
       </x:c>
-      <x:c r="B3" s="44" t="str">
+      <x:c r="B3" s="52" t="str">
         <x:v>#2</x:v>
       </x:c>
-      <x:c r="C3" s="44" t="str">
+      <x:c r="C3" s="52" t="str">
         <x:v>Melhoria</x:v>
       </x:c>
-      <x:c r="D3" s="44" t="str">
+      <x:c r="D3" s="52" t="str">
         <x:v>Baixa</x:v>
       </x:c>
-      <x:c r="E3" s="44" t="str">
+      <x:c r="E3" s="52" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="F3" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G3" s="44" t="str">
+      <x:c r="F3" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G3" s="52" t="str">
         <x:v>GET</x:v>
       </x:c>
-      <x:c r="H3" s="44" t="str">
+      <x:c r="H3" s="52" t="str">
         <x:v>Restrições</x:v>
       </x:c>
-      <x:c r="I3" s="44" t="str">
+      <x:c r="I3" s="52" t="str">
         <x:v>Proibir busca de CPF com mais de 11 dígitos</x:v>
       </x:c>
-      <x:c r="J3" s="44" t="str">
+      <x:c r="J3" s="52" t="str">
         <x:v>Ao tentar utilizar a função de procurar CPF com restrições, a API aceita qualquer tamanho de CPF como instrução, para economizar tempo e recursos, o ideal seria que ele apenas aceitasse requisições de CPFs apenas com 11 dígitos.</x:v>
       </x:c>
-      <x:c r="K3" s="44" t="str">
+      <x:c r="K3" s="52" t="str">
         <x:v>Rejeitar CPF com mais de 11 dígitos e retornar validação clara.</x:v>
       </x:c>
-      <x:c r="L3" s="44" t="str">
+      <x:c r="L3" s="52" t="str">
         <x:v>Reduz precisão das validações e da comunicação da API para cenários de consulta.</x:v>
       </x:c>
-      <x:c r="M3" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N3" s="44" t="str">
-        <x:v>GET, Melhoria, Restrições</x:v>
-      </x:c>
-      <x:c r="O3" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="64.5" customHeight="1">
-      <x:c r="A4" s="43" t="str">
+      <x:c r="M3"/>
+      <x:c r="N3"/>
+      <x:c r="O3"/>
+    </x:row>
+    <x:row r="4" ht="84" customHeight="1">
+      <x:c r="A4" s="52" t="str">
         <x:v>BUG-003</x:v>
       </x:c>
-      <x:c r="B4" s="44" t="str">
+      <x:c r="B4" s="52" t="str">
         <x:v>#3</x:v>
       </x:c>
-      <x:c r="C4" s="44" t="str">
+      <x:c r="C4" s="52" t="str">
         <x:v>Melhoria</x:v>
       </x:c>
-      <x:c r="D4" s="44" t="str">
+      <x:c r="D4" s="52" t="str">
         <x:v>Baixa</x:v>
       </x:c>
-      <x:c r="E4" s="44" t="str">
+      <x:c r="E4" s="52" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="F4" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G4" s="44" t="str">
+      <x:c r="F4" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G4" s="52" t="str">
         <x:v>GET</x:v>
       </x:c>
-      <x:c r="H4" s="44" t="str">
+      <x:c r="H4" s="52" t="str">
         <x:v>Restrições</x:v>
       </x:c>
-      <x:c r="I4" s="44" t="str">
+      <x:c r="I4" s="52" t="str">
         <x:v>Proibir busca de CPF enviando letras no lugar de números</x:v>
       </x:c>
-      <x:c r="J4" s="44" t="str">
+      <x:c r="J4" s="52" t="str">
         <x:v>Ao tentar utilizar a função de procurar CPF com restrições, a API aceita qualquer caractere como instrução, para economizar tempo e recursos, o ideal seria que ele apenas aceitasse requisições utilizando apenas números.</x:v>
       </x:c>
-      <x:c r="K4" s="44" t="str">
+      <x:c r="K4" s="52" t="str">
         <x:v>Aceitar apenas CPF numérico no formato esperado pela API.</x:v>
       </x:c>
-      <x:c r="L4" s="44" t="str">
+      <x:c r="L4" s="52" t="str">
         <x:v>Reduz precisão das validações e da comunicação da API para cenários de consulta.</x:v>
       </x:c>
-      <x:c r="M4" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N4" s="44" t="str">
-        <x:v>GET, Melhoria, Restrições</x:v>
-      </x:c>
-      <x:c r="O4" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="64.5" customHeight="1">
-      <x:c r="A5" s="43" t="str">
+      <x:c r="M4"/>
+      <x:c r="N4"/>
+      <x:c r="O4"/>
+    </x:row>
+    <x:row r="5" ht="84" customHeight="1">
+      <x:c r="A5" s="52" t="str">
         <x:v>BUG-004</x:v>
       </x:c>
-      <x:c r="B5" s="44" t="str">
+      <x:c r="B5" s="52" t="str">
         <x:v>#4</x:v>
       </x:c>
-      <x:c r="C5" s="44" t="str">
+      <x:c r="C5" s="52" t="str">
         <x:v>Regra de negócio</x:v>
       </x:c>
-      <x:c r="D5" s="44" t="str">
+      <x:c r="D5" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E5" s="44" t="str">
+      <x:c r="E5" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F5" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G5" s="44" t="str">
+      <x:c r="F5" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G5" s="52" t="str">
         <x:v>GET</x:v>
       </x:c>
-      <x:c r="H5" s="44" t="str">
+      <x:c r="H5" s="52" t="str">
         <x:v>Restrições</x:v>
       </x:c>
-      <x:c r="I5" s="44" t="str">
+      <x:c r="I5" s="52" t="str">
         <x:v>Correção de mensagem de resposta para o GET de CPF restrito</x:v>
       </x:c>
-      <x:c r="J5" s="44" t="str">
+      <x:c r="J5" s="52" t="str">
         <x:v>Ao procurar um CPF que possui restrição, a mensagem recebida pelo response body deve ter um formato como especificado na documentação.</x:v>
       </x:c>
-      <x:c r="K5" s="44" t="str">
+      <x:c r="K5" s="52" t="str">
         <x:v>Aplicar a regra de restrição de CPF e retornar mensagem no padrão documentado.</x:v>
       </x:c>
-      <x:c r="L5" s="44" t="str">
+      <x:c r="L5" s="52" t="str">
         <x:v>Reduz precisão das validações e da comunicação da API para cenários de consulta.</x:v>
       </x:c>
-      <x:c r="M5" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N5" s="44" t="str">
-        <x:v>GET, Regra de negócio, Restrições</x:v>
-      </x:c>
-      <x:c r="O5" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="64.5" customHeight="1">
-      <x:c r="A6" s="43" t="str">
+      <x:c r="M5"/>
+      <x:c r="N5"/>
+      <x:c r="O5"/>
+    </x:row>
+    <x:row r="6" ht="84" customHeight="1">
+      <x:c r="A6" s="52" t="str">
         <x:v>BUG-005</x:v>
       </x:c>
-      <x:c r="B6" s="44" t="str">
+      <x:c r="B6" s="52" t="str">
         <x:v>#5</x:v>
       </x:c>
-      <x:c r="C6" s="44" t="str">
+      <x:c r="C6" s="52" t="str">
         <x:v>Melhoria</x:v>
       </x:c>
-      <x:c r="D6" s="44" t="str">
+      <x:c r="D6" s="52" t="str">
         <x:v>Baixa</x:v>
       </x:c>
-      <x:c r="E6" s="44" t="str">
+      <x:c r="E6" s="52" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="F6" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G6" s="44" t="str">
+      <x:c r="F6" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G6" s="52" t="str">
         <x:v>GET</x:v>
       </x:c>
-      <x:c r="H6" s="44" t="str">
+      <x:c r="H6" s="52" t="str">
         <x:v>Restrições</x:v>
       </x:c>
-      <x:c r="I6" s="44" t="str">
+      <x:c r="I6" s="52" t="str">
         <x:v>Mostrar no GET de simulações que o CPF possui restrição</x:v>
       </x:c>
-      <x:c r="J6" s="44" t="str">
+      <x:c r="J6" s="52" t="str">
         <x:v>Ao utilizar o GET de simulações, seria interessante se o usuário fosse informado caso seu CPF tenha algum tipo de restrição.</x:v>
       </x:c>
-      <x:c r="K6" s="44" t="str">
+      <x:c r="K6" s="52" t="str">
         <x:v>Aplicar a regra de restrição de CPF e retornar mensagem no padrão documentado.</x:v>
       </x:c>
-      <x:c r="L6" s="44" t="str">
+      <x:c r="L6" s="52" t="str">
         <x:v>Reduz precisão das validações e da comunicação da API para cenários de consulta.</x:v>
       </x:c>
-      <x:c r="M6" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N6" s="44" t="str">
-        <x:v>GET, Melhoria, Simulações</x:v>
-      </x:c>
-      <x:c r="O6" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="64.5" customHeight="1">
-      <x:c r="A7" s="43" t="str">
+      <x:c r="M6"/>
+      <x:c r="N6"/>
+      <x:c r="O6"/>
+    </x:row>
+    <x:row r="7" ht="84" customHeight="1">
+      <x:c r="A7" s="52" t="str">
         <x:v>BUG-006</x:v>
       </x:c>
-      <x:c r="B7" s="44" t="str">
+      <x:c r="B7" s="52" t="str">
         <x:v>#6</x:v>
       </x:c>
-      <x:c r="C7" s="44" t="str">
+      <x:c r="C7" s="52" t="str">
         <x:v>Regra de negócio</x:v>
       </x:c>
-      <x:c r="D7" s="44" t="str">
+      <x:c r="D7" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E7" s="44" t="str">
+      <x:c r="E7" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F7" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G7" s="44" t="str">
+      <x:c r="F7" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G7" s="52" t="str">
         <x:v>GET</x:v>
       </x:c>
-      <x:c r="H7" s="44" t="str">
+      <x:c r="H7" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I7" s="44" t="str">
+      <x:c r="I7" s="52" t="str">
         <x:v>Correção status code de simulações ao verificar lista vazia</x:v>
       </x:c>
-      <x:c r="J7" s="44" t="str">
+      <x:c r="J7" s="52" t="str">
         <x:v>Ao verificar a lista geral de simulações e não existir nenhum conteúdo na lista, o status code esperado deve ser 204 e não 200 como recebido.</x:v>
       </x:c>
-      <x:c r="K7" s="44" t="str">
+      <x:c r="K7" s="52" t="str">
         <x:v>Retornar 204 quando não houver simulações cadastradas.</x:v>
       </x:c>
-      <x:c r="L7" s="44" t="str">
+      <x:c r="L7" s="52" t="str">
         <x:v>Reduz precisão das validações e da comunicação da API para cenários de consulta.</x:v>
       </x:c>
-      <x:c r="M7" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N7" s="44" t="str">
-        <x:v>GET, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O7" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="64.5" customHeight="1">
-      <x:c r="A8" s="43" t="str">
+      <x:c r="M7"/>
+      <x:c r="N7"/>
+      <x:c r="O7"/>
+    </x:row>
+    <x:row r="8" ht="84" customHeight="1">
+      <x:c r="A8" s="52" t="str">
         <x:v>BUG-007</x:v>
       </x:c>
-      <x:c r="B8" s="44" t="str">
+      <x:c r="B8" s="52" t="str">
         <x:v>#7</x:v>
       </x:c>
-      <x:c r="C8" s="44" t="str">
+      <x:c r="C8" s="52" t="str">
         <x:v>Regra de negócio</x:v>
       </x:c>
-      <x:c r="D8" s="44" t="str">
+      <x:c r="D8" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E8" s="44" t="str">
+      <x:c r="E8" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F8" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G8" s="44" t="str">
+      <x:c r="F8" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G8" s="52" t="str">
         <x:v>DELETE</x:v>
       </x:c>
-      <x:c r="H8" s="44" t="str">
+      <x:c r="H8" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I8" s="44" t="str">
+      <x:c r="I8" s="52" t="str">
         <x:v>Correção de status code ao tentar excluir simulação inexistente</x:v>
       </x:c>
-      <x:c r="J8" s="44" t="str">
+      <x:c r="J8" s="52" t="str">
         <x:v>Ao tentar excluir simulação inexistente um status code de 404 é esperado, porém um status de 200 é recebido.</x:v>
       </x:c>
-      <x:c r="K8" s="44" t="str">
+      <x:c r="K8" s="52" t="str">
         <x:v>Retornar 404 e mensagem informando que a simulação não foi encontrada.</x:v>
       </x:c>
-      <x:c r="L8" s="44" t="str">
+      <x:c r="L8" s="52" t="str">
         <x:v>Pode induzir o consumidor da API a interpretar exclusões inexistentes como sucesso.</x:v>
       </x:c>
-      <x:c r="M8" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N8" s="44" t="str">
-        <x:v>DELETE, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O8" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="64.5" customHeight="1">
-      <x:c r="A9" s="43" t="str">
+      <x:c r="M8"/>
+      <x:c r="N8"/>
+      <x:c r="O8"/>
+    </x:row>
+    <x:row r="9" ht="84" customHeight="1">
+      <x:c r="A9" s="52" t="str">
         <x:v>BUG-008</x:v>
       </x:c>
-      <x:c r="B9" s="44" t="str">
+      <x:c r="B9" s="52" t="str">
         <x:v>#8</x:v>
       </x:c>
-      <x:c r="C9" s="44" t="str">
+      <x:c r="C9" s="52" t="str">
         <x:v>Regra de negócio</x:v>
       </x:c>
-      <x:c r="D9" s="44" t="str">
+      <x:c r="D9" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E9" s="44" t="str">
+      <x:c r="E9" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F9" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G9" s="44" t="str">
+      <x:c r="F9" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G9" s="52" t="str">
         <x:v>DELETE</x:v>
       </x:c>
-      <x:c r="H9" s="44" t="str">
+      <x:c r="H9" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I9" s="44" t="str">
+      <x:c r="I9" s="52" t="str">
         <x:v>Correção de mensagem ao tentar excluir simulação inexistente</x:v>
       </x:c>
-      <x:c r="J9" s="44" t="str">
+      <x:c r="J9" s="52" t="str">
         <x:v>Ao tentar excluir simulação inexistente uma mensagem informando que a simulação não foi encontrada é esperada.</x:v>
       </x:c>
-      <x:c r="K9" s="44" t="str">
+      <x:c r="K9" s="52" t="str">
         <x:v>Retornar 404 e mensagem informando que a simulação não foi encontrada.</x:v>
       </x:c>
-      <x:c r="L9" s="44" t="str">
+      <x:c r="L9" s="52" t="str">
         <x:v>Pode induzir o consumidor da API a interpretar exclusões inexistentes como sucesso.</x:v>
       </x:c>
-      <x:c r="M9" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N9" s="44" t="str">
-        <x:v>DELETE, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O9" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="64.5" customHeight="1">
-      <x:c r="A10" s="43" t="str">
+      <x:c r="M9"/>
+      <x:c r="N9"/>
+      <x:c r="O9"/>
+    </x:row>
+    <x:row r="10" ht="84" customHeight="1">
+      <x:c r="A10" s="52" t="str">
         <x:v>BUG-009</x:v>
       </x:c>
-      <x:c r="B10" s="44" t="str">
+      <x:c r="B10" s="52" t="str">
         <x:v>#9</x:v>
       </x:c>
-      <x:c r="C10" s="44" t="str">
+      <x:c r="C10" s="52" t="str">
         <x:v>Regra de negócio</x:v>
       </x:c>
-      <x:c r="D10" s="44" t="str">
+      <x:c r="D10" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E10" s="44" t="str">
+      <x:c r="E10" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F10" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G10" s="44" t="str">
+      <x:c r="F10" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G10" s="52" t="str">
         <x:v>DELETE</x:v>
       </x:c>
-      <x:c r="H10" s="44" t="str">
+      <x:c r="H10" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I10" s="44" t="str">
+      <x:c r="I10" s="52" t="str">
         <x:v>Correção de status code ao deletar uma simulação com sucesso</x:v>
       </x:c>
-      <x:c r="J10" s="44" t="str">
+      <x:c r="J10" s="52" t="str">
         <x:v>Ao excluir uma simulação com sucesso, é esperado que um status code específico seja devolvido.</x:v>
       </x:c>
-      <x:c r="K10" s="44" t="str">
+      <x:c r="K10" s="52" t="str">
         <x:v>Retornar o status code esperado para exclusão realizada com sucesso.</x:v>
       </x:c>
-      <x:c r="L10" s="44" t="str">
+      <x:c r="L10" s="52" t="str">
         <x:v>Pode induzir o consumidor da API a interpretar exclusões inexistentes como sucesso.</x:v>
       </x:c>
-      <x:c r="M10" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N10" s="44" t="str">
-        <x:v>DELETE, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O10" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="64.5" customHeight="1">
-      <x:c r="A11" s="43" t="str">
+      <x:c r="M10"/>
+      <x:c r="N10"/>
+      <x:c r="O10"/>
+    </x:row>
+    <x:row r="11" ht="84" customHeight="1">
+      <x:c r="A11" s="52" t="str">
         <x:v>BUG-010</x:v>
       </x:c>
-      <x:c r="B11" s="44" t="str">
+      <x:c r="B11" s="52" t="str">
         <x:v>#10</x:v>
       </x:c>
-      <x:c r="C11" s="44" t="str">
+      <x:c r="C11" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D11" s="44" t="str">
+      <x:c r="D11" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E11" s="44" t="str">
+      <x:c r="E11" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F11" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G11" s="44" t="str">
+      <x:c r="F11" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G11" s="52" t="str">
         <x:v>PUT</x:v>
       </x:c>
-      <x:c r="H11" s="44" t="str">
+      <x:c r="H11" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I11" s="44" t="str">
+      <x:c r="I11" s="52" t="str">
         <x:v>Proibir atualização de cadastro deixando CPF vazio</x:v>
       </x:c>
-      <x:c r="J11" s="44" t="str">
+      <x:c r="J11" s="52" t="str">
         <x:v>Ao tentar atualizar um cadastro deixando o campo CPF vazio ele aceita e atualiza o cadastro ao invés de negar.</x:v>
       </x:c>
-      <x:c r="K11" s="44" t="str">
+      <x:c r="K11" s="52" t="str">
         <x:v>Negar operação quando CPF obrigatório estiver vazio ou ausente.</x:v>
       </x:c>
-      <x:c r="L11" s="44" t="str">
+      <x:c r="L11" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M11" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N11" s="44" t="str">
-        <x:v>Bug, PUT, Simulações</x:v>
-      </x:c>
-      <x:c r="O11" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="64.5" customHeight="1">
-      <x:c r="A12" s="43" t="str">
+      <x:c r="M11"/>
+      <x:c r="N11"/>
+      <x:c r="O11"/>
+    </x:row>
+    <x:row r="12" ht="84" customHeight="1">
+      <x:c r="A12" s="52" t="str">
         <x:v>BUG-011</x:v>
       </x:c>
-      <x:c r="B12" s="44" t="str">
+      <x:c r="B12" s="52" t="str">
         <x:v>#11</x:v>
       </x:c>
-      <x:c r="C12" s="44" t="str">
+      <x:c r="C12" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D12" s="44" t="str">
+      <x:c r="D12" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E12" s="44" t="str">
+      <x:c r="E12" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F12" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G12" s="44" t="str">
+      <x:c r="F12" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G12" s="52" t="str">
         <x:v>PUT</x:v>
       </x:c>
-      <x:c r="H12" s="44" t="str">
+      <x:c r="H12" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I12" s="44" t="str">
+      <x:c r="I12" s="52" t="str">
         <x:v>Proibir atualização de cadastro deixando o campo nome vazio</x:v>
       </x:c>
-      <x:c r="J12" s="44" t="str">
+      <x:c r="J12" s="52" t="str">
         <x:v>Ao tentar atualizar um cadastro deixando o campo nome vazio ele aceita e atualiza o cadastro ao invés de negar.</x:v>
       </x:c>
-      <x:c r="K12" s="44" t="str">
+      <x:c r="K12" s="52" t="str">
         <x:v>Negar operação quando nome obrigatório estiver vazio ou ausente.</x:v>
       </x:c>
-      <x:c r="L12" s="44" t="str">
+      <x:c r="L12" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M12" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N12" s="44" t="str">
-        <x:v>Bug, PUT, Simulações</x:v>
-      </x:c>
-      <x:c r="O12" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="64.5" customHeight="1">
-      <x:c r="A13" s="43" t="str">
+      <x:c r="M12"/>
+      <x:c r="N12"/>
+      <x:c r="O12"/>
+    </x:row>
+    <x:row r="13" ht="84" customHeight="1">
+      <x:c r="A13" s="52" t="str">
         <x:v>BUG-012</x:v>
       </x:c>
-      <x:c r="B13" s="44" t="str">
+      <x:c r="B13" s="52" t="str">
         <x:v>#12</x:v>
       </x:c>
-      <x:c r="C13" s="44" t="str">
+      <x:c r="C13" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D13" s="44" t="str">
+      <x:c r="D13" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E13" s="44" t="str">
+      <x:c r="E13" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F13" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G13" s="44" t="str">
+      <x:c r="F13" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G13" s="52" t="str">
         <x:v>PUT</x:v>
       </x:c>
-      <x:c r="H13" s="44" t="str">
+      <x:c r="H13" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I13" s="44" t="str">
+      <x:c r="I13" s="52" t="str">
         <x:v>Correção de bug de atualização - corrigir campo valor de atualização que não está sendo alterado</x:v>
       </x:c>
-      <x:c r="J13" s="44" t="str">
+      <x:c r="J13" s="52" t="str">
         <x:v>Ao tentar atualizar o campo valor em um cadastro de simulação, ele não está sendo devidamente atualizado.</x:v>
       </x:c>
-      <x:c r="K13" s="44" t="str">
+      <x:c r="K13" s="52" t="str">
         <x:v>Atualizar corretamente o valor informado no cadastro de simulação.</x:v>
       </x:c>
-      <x:c r="L13" s="44" t="str">
+      <x:c r="L13" s="52" t="str">
         <x:v>Afeta aderência às regras de negócio e previsibilidade do contrato da API.</x:v>
       </x:c>
-      <x:c r="M13" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N13" s="44" t="str">
-        <x:v>Bug, PUT, Simulações</x:v>
-      </x:c>
-      <x:c r="O13" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="64.5" customHeight="1">
-      <x:c r="A14" s="43" t="str">
+      <x:c r="M13"/>
+      <x:c r="N13"/>
+      <x:c r="O13"/>
+    </x:row>
+    <x:row r="14" ht="84" customHeight="1">
+      <x:c r="A14" s="52" t="str">
         <x:v>BUG-013</x:v>
       </x:c>
-      <x:c r="B14" s="44" t="str">
+      <x:c r="B14" s="52" t="str">
         <x:v>#13</x:v>
       </x:c>
-      <x:c r="C14" s="44" t="str">
+      <x:c r="C14" s="52" t="str">
         <x:v>Regra de negócio</x:v>
       </x:c>
-      <x:c r="D14" s="44" t="str">
+      <x:c r="D14" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E14" s="44" t="str">
+      <x:c r="E14" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F14" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G14" s="44" t="str">
+      <x:c r="F14" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G14" s="52" t="str">
         <x:v>PUT</x:v>
       </x:c>
-      <x:c r="H14" s="44" t="str">
+      <x:c r="H14" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I14" s="44" t="str">
+      <x:c r="I14" s="52" t="str">
         <x:v>Correção de mensagem de retorno ao atualizar CPF já existente</x:v>
       </x:c>
-      <x:c r="J14" s="44" t="str">
+      <x:c r="J14" s="52" t="str">
         <x:v>Ao tentar atualizar um cadastro utilizando o CPF de outra simulação, uma mensagem específica é esperada e não é recebida em retorno.</x:v>
       </x:c>
-      <x:c r="K14" s="44" t="str">
+      <x:c r="K14" s="52" t="str">
         <x:v>Comportamento deve seguir a regra de negócio e a documentação da API.</x:v>
       </x:c>
-      <x:c r="L14" s="44" t="str">
+      <x:c r="L14" s="52" t="str">
         <x:v>Afeta aderência às regras de negócio e previsibilidade do contrato da API.</x:v>
       </x:c>
-      <x:c r="M14" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N14" s="44" t="str">
-        <x:v>PUT, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O14" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="64.5" customHeight="1">
-      <x:c r="A15" s="43" t="str">
+      <x:c r="M14"/>
+      <x:c r="N14"/>
+      <x:c r="O14"/>
+    </x:row>
+    <x:row r="15" ht="84" customHeight="1">
+      <x:c r="A15" s="52" t="str">
         <x:v>BUG-014</x:v>
       </x:c>
-      <x:c r="B15" s="44" t="str">
+      <x:c r="B15" s="52" t="str">
         <x:v>#14</x:v>
       </x:c>
-      <x:c r="C15" s="44" t="str">
+      <x:c r="C15" s="52" t="str">
         <x:v>Regra de negócio</x:v>
       </x:c>
-      <x:c r="D15" s="44" t="str">
+      <x:c r="D15" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E15" s="44" t="str">
+      <x:c r="E15" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F15" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G15" s="44" t="str">
+      <x:c r="F15" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G15" s="52" t="str">
         <x:v>PUT</x:v>
       </x:c>
-      <x:c r="H15" s="44" t="str">
+      <x:c r="H15" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I15" s="44" t="str">
+      <x:c r="I15" s="52" t="str">
         <x:v>Correção de status code de atualização utilizando CPF duplicado</x:v>
       </x:c>
-      <x:c r="J15" s="44" t="str">
+      <x:c r="J15" s="52" t="str">
         <x:v>Ao tentar atualizar um cadastro utilizando o CPF de outra simulação, um status code específico é esperada e não é recebido em retorno.</x:v>
       </x:c>
-      <x:c r="K15" s="44" t="str">
+      <x:c r="K15" s="52" t="str">
         <x:v>Retornar status code e mensagem específicos para CPF já cadastrado.</x:v>
       </x:c>
-      <x:c r="L15" s="44" t="str">
+      <x:c r="L15" s="52" t="str">
         <x:v>Afeta aderência às regras de negócio e previsibilidade do contrato da API.</x:v>
       </x:c>
-      <x:c r="M15" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N15" s="44" t="str">
-        <x:v>PUT, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O15" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="64.5" customHeight="1">
-      <x:c r="A16" s="43" t="str">
+      <x:c r="M15"/>
+      <x:c r="N15"/>
+      <x:c r="O15"/>
+    </x:row>
+    <x:row r="16" ht="84" customHeight="1">
+      <x:c r="A16" s="52" t="str">
         <x:v>BUG-015</x:v>
       </x:c>
-      <x:c r="B16" s="44" t="str">
+      <x:c r="B16" s="52" t="str">
         <x:v>#15</x:v>
       </x:c>
-      <x:c r="C16" s="44" t="str">
+      <x:c r="C16" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D16" s="44" t="str">
+      <x:c r="D16" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E16" s="44" t="str">
+      <x:c r="E16" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F16" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G16" s="44" t="str">
+      <x:c r="F16" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G16" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H16" s="44" t="str">
+      <x:c r="H16" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I16" s="44" t="str">
+      <x:c r="I16" s="52" t="str">
         <x:v>Proibir a atualização de cadastro através do POST</x:v>
       </x:c>
-      <x:c r="J16" s="44" t="str">
+      <x:c r="J16" s="52" t="str">
         <x:v>Ao enviar no request body um corpo contendo o campo ID de um usuário cadastrado, ao invés de tentar realizar um novo cadastro e alterar o ID ele altera as informações do usuário que já foi cadastrado mantendo o ID informado.</x:v>
       </x:c>
-      <x:c r="K16" s="44" t="str">
+      <x:c r="K16" s="52" t="str">
         <x:v>POST deve criar novo recurso, sem alterar simulação existente por ID enviado no corpo.</x:v>
       </x:c>
-      <x:c r="L16" s="44" t="str">
+      <x:c r="L16" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M16" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N16" s="44" t="str">
-        <x:v>Bug, POST, Simulações</x:v>
-      </x:c>
-      <x:c r="O16" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="64.5" customHeight="1">
-      <x:c r="A17" s="43" t="str">
+      <x:c r="M16"/>
+      <x:c r="N16"/>
+      <x:c r="O16"/>
+    </x:row>
+    <x:row r="17" ht="84" customHeight="1">
+      <x:c r="A17" s="52" t="str">
         <x:v>BUG-016</x:v>
       </x:c>
-      <x:c r="B17" s="44" t="str">
+      <x:c r="B17" s="52" t="str">
         <x:v>#16</x:v>
       </x:c>
-      <x:c r="C17" s="44" t="str">
+      <x:c r="C17" s="52" t="str">
         <x:v>Melhoria</x:v>
       </x:c>
-      <x:c r="D17" s="44" t="str">
+      <x:c r="D17" s="52" t="str">
         <x:v>Baixa</x:v>
       </x:c>
-      <x:c r="E17" s="44" t="str">
+      <x:c r="E17" s="52" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="F17" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G17" s="44" t="str">
+      <x:c r="F17" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G17" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H17" s="44" t="str">
+      <x:c r="H17" s="52" t="str">
         <x:v>Restrições</x:v>
       </x:c>
-      <x:c r="I17" s="44" t="str">
+      <x:c r="I17" s="52" t="str">
         <x:v>Proibir o cadastro de simulações que possuem restrições no CPF</x:v>
       </x:c>
-      <x:c r="J17" s="44" t="str">
+      <x:c r="J17" s="52" t="str">
         <x:v>Ao tentar cadastrar uma simulação utilizando um dos CPFs com restrição, ele aceita normalmente.</x:v>
       </x:c>
-      <x:c r="K17" s="44" t="str">
+      <x:c r="K17" s="52" t="str">
         <x:v>Comportamento deve seguir a regra de negócio e a documentação da API.</x:v>
       </x:c>
-      <x:c r="L17" s="44" t="str">
+      <x:c r="L17" s="52" t="str">
         <x:v>Melhora clareza da resposta e previsibilidade da integração.</x:v>
       </x:c>
-      <x:c r="M17" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N17" s="44" t="str">
-        <x:v>Melhoria, POST, Simulações</x:v>
-      </x:c>
-      <x:c r="O17" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="64.5" customHeight="1">
-      <x:c r="A18" s="43" t="str">
+      <x:c r="M17"/>
+      <x:c r="N17"/>
+      <x:c r="O17"/>
+    </x:row>
+    <x:row r="18" ht="84" customHeight="1">
+      <x:c r="A18" s="52" t="str">
         <x:v>BUG-017</x:v>
       </x:c>
-      <x:c r="B18" s="44" t="str">
+      <x:c r="B18" s="52" t="str">
         <x:v>#17</x:v>
       </x:c>
-      <x:c r="C18" s="44" t="str">
+      <x:c r="C18" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D18" s="44" t="str">
+      <x:c r="D18" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E18" s="44" t="str">
+      <x:c r="E18" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F18" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G18" s="44" t="str">
+      <x:c r="F18" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G18" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H18" s="44" t="str">
+      <x:c r="H18" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I18" s="44" t="str">
+      <x:c r="I18" s="52" t="str">
         <x:v>Proibir o cadastro enviando letras no lugar de números do CPF</x:v>
       </x:c>
-      <x:c r="J18" s="44" t="str">
+      <x:c r="J18" s="52" t="str">
         <x:v>Ao tentar cadastrar uma nova simulação, foi possível realizar o cadastro informando letras no lugar do CPF com números.</x:v>
       </x:c>
-      <x:c r="K18" s="44" t="str">
+      <x:c r="K18" s="52" t="str">
         <x:v>Aceitar apenas CPF numérico no formato esperado pela API.</x:v>
       </x:c>
-      <x:c r="L18" s="44" t="str">
+      <x:c r="L18" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M18" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N18" s="44" t="str">
-        <x:v>Bug, POST, Simulações</x:v>
-      </x:c>
-      <x:c r="O18" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="64.5" customHeight="1">
-      <x:c r="A19" s="43" t="str">
+      <x:c r="M18"/>
+      <x:c r="N18"/>
+      <x:c r="O18"/>
+    </x:row>
+    <x:row r="19" ht="84" customHeight="1">
+      <x:c r="A19" s="52" t="str">
         <x:v>BUG-018</x:v>
       </x:c>
-      <x:c r="B19" s="44" t="str">
+      <x:c r="B19" s="52" t="str">
         <x:v>#18</x:v>
       </x:c>
-      <x:c r="C19" s="44" t="str">
+      <x:c r="C19" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D19" s="44" t="str">
+      <x:c r="D19" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E19" s="44" t="str">
+      <x:c r="E19" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F19" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G19" s="44" t="str">
+      <x:c r="F19" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G19" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H19" s="44" t="str">
+      <x:c r="H19" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I19" s="44" t="str">
+      <x:c r="I19" s="52" t="str">
         <x:v>Proibir o cadastro enviando CPF menor que onze digitos</x:v>
       </x:c>
-      <x:c r="J19" s="44" t="str">
+      <x:c r="J19" s="52" t="str">
         <x:v>Ao tentar cadastrar uma nova simulação, foi possível realizar o cadastro informando menos de 11 dígitos do CPF.</x:v>
       </x:c>
-      <x:c r="K19" s="44" t="str">
+      <x:c r="K19" s="52" t="str">
         <x:v>Rejeitar CPF com menos de 11 dígitos e retornar validação clara.</x:v>
       </x:c>
-      <x:c r="L19" s="44" t="str">
+      <x:c r="L19" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M19" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N19" s="44" t="str">
-        <x:v>Bug, POST, Simulações</x:v>
-      </x:c>
-      <x:c r="O19" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="64.5" customHeight="1">
-      <x:c r="A20" s="43" t="str">
+      <x:c r="M19"/>
+      <x:c r="N19"/>
+      <x:c r="O19"/>
+    </x:row>
+    <x:row r="20" ht="84" customHeight="1">
+      <x:c r="A20" s="52" t="str">
         <x:v>BUG-019</x:v>
       </x:c>
-      <x:c r="B20" s="44" t="str">
+      <x:c r="B20" s="52" t="str">
         <x:v>#19</x:v>
       </x:c>
-      <x:c r="C20" s="44" t="str">
+      <x:c r="C20" s="52" t="str">
         <x:v>Regra de negócio</x:v>
       </x:c>
-      <x:c r="D20" s="44" t="str">
+      <x:c r="D20" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E20" s="44" t="str">
+      <x:c r="E20" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F20" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G20" s="44" t="str">
+      <x:c r="F20" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G20" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H20" s="44" t="str">
+      <x:c r="H20" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I20" s="44" t="str">
+      <x:c r="I20" s="52" t="str">
         <x:v>Correção de mensagem de retorno de cadastro de CPF duplicado</x:v>
       </x:c>
-      <x:c r="J20" s="44" t="str">
+      <x:c r="J20" s="52" t="str">
         <x:v>Ao tentar cadastrar uma simulação utilizando um CPF já existente, uma mensagem específica de retorno é esperada.</x:v>
       </x:c>
-      <x:c r="K20" s="44" t="str">
+      <x:c r="K20" s="52" t="str">
         <x:v>Retornar status code e mensagem específicos para CPF já cadastrado.</x:v>
       </x:c>
-      <x:c r="L20" s="44" t="str">
+      <x:c r="L20" s="52" t="str">
         <x:v>Afeta aderência às regras de negócio e previsibilidade do contrato da API.</x:v>
       </x:c>
-      <x:c r="M20" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N20" s="44" t="str">
-        <x:v>POST, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O20" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="64.5" customHeight="1">
-      <x:c r="A21" s="43" t="str">
+      <x:c r="M20"/>
+      <x:c r="N20"/>
+      <x:c r="O20"/>
+    </x:row>
+    <x:row r="21" ht="84" customHeight="1">
+      <x:c r="A21" s="52" t="str">
         <x:v>BUG-020</x:v>
       </x:c>
-      <x:c r="B21" s="44" t="str">
+      <x:c r="B21" s="52" t="str">
         <x:v>#20</x:v>
       </x:c>
-      <x:c r="C21" s="44" t="str">
+      <x:c r="C21" s="52" t="str">
         <x:v>Regra de negócio</x:v>
       </x:c>
-      <x:c r="D21" s="44" t="str">
+      <x:c r="D21" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E21" s="44" t="str">
+      <x:c r="E21" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F21" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G21" s="44" t="str">
+      <x:c r="F21" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G21" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H21" s="44" t="str">
+      <x:c r="H21" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I21" s="44" t="str">
+      <x:c r="I21" s="52" t="str">
         <x:v>Correção de status code de cadastro de CPF duplicado</x:v>
       </x:c>
-      <x:c r="J21" s="44" t="str">
+      <x:c r="J21" s="52" t="str">
         <x:v>Ao tentar cadastrar uma simulação utilizando um CPF já existente, um status code específico de retorno é esperado.</x:v>
       </x:c>
-      <x:c r="K21" s="44" t="str">
+      <x:c r="K21" s="52" t="str">
         <x:v>Retornar status code e mensagem específicos para CPF já cadastrado.</x:v>
       </x:c>
-      <x:c r="L21" s="44" t="str">
+      <x:c r="L21" s="52" t="str">
         <x:v>Afeta aderência às regras de negócio e previsibilidade do contrato da API.</x:v>
       </x:c>
-      <x:c r="M21" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N21" s="44" t="str">
-        <x:v>POST, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O21" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="64.5" customHeight="1">
-      <x:c r="A22" s="43" t="str">
+      <x:c r="M21"/>
+      <x:c r="N21"/>
+      <x:c r="O21"/>
+    </x:row>
+    <x:row r="22" ht="84" customHeight="1">
+      <x:c r="A22" s="52" t="str">
         <x:v>BUG-021</x:v>
       </x:c>
-      <x:c r="B22" s="44" t="str">
+      <x:c r="B22" s="52" t="str">
         <x:v>#21</x:v>
       </x:c>
-      <x:c r="C22" s="44" t="str">
+      <x:c r="C22" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D22" s="44" t="str">
+      <x:c r="D22" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E22" s="44" t="str">
+      <x:c r="E22" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F22" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G22" s="44" t="str">
+      <x:c r="F22" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G22" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H22" s="44" t="str">
+      <x:c r="H22" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I22" s="44" t="str">
+      <x:c r="I22" s="52" t="str">
         <x:v>Proibir o cadastro sem enviar nenhum CPF</x:v>
       </x:c>
-      <x:c r="J22" s="44" t="str">
+      <x:c r="J22" s="52" t="str">
         <x:v>Ao não enviar o campo de CPF no cadastro, é esperado que o cadastro seja negado, porém, ele aceita e cadastra a simulação mesmo assim.</x:v>
       </x:c>
-      <x:c r="K22" s="44" t="str">
+      <x:c r="K22" s="52" t="str">
         <x:v>Negar cadastro sem CPF e retornar validação clara.</x:v>
       </x:c>
-      <x:c r="L22" s="44" t="str">
+      <x:c r="L22" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M22" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N22" s="44" t="str">
-        <x:v>Bug, POST, Simulações</x:v>
-      </x:c>
-      <x:c r="O22" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="64.5" customHeight="1">
-      <x:c r="A23" s="43" t="str">
+      <x:c r="M22"/>
+      <x:c r="N22"/>
+      <x:c r="O22"/>
+    </x:row>
+    <x:row r="23" ht="84" customHeight="1">
+      <x:c r="A23" s="52" t="str">
         <x:v>BUG-022</x:v>
       </x:c>
-      <x:c r="B23" s="44" t="str">
+      <x:c r="B23" s="52" t="str">
         <x:v>#22</x:v>
       </x:c>
-      <x:c r="C23" s="44" t="str">
+      <x:c r="C23" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D23" s="44" t="str">
+      <x:c r="D23" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E23" s="44" t="str">
+      <x:c r="E23" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F23" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G23" s="44" t="str">
+      <x:c r="F23" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G23" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H23" s="44" t="str">
+      <x:c r="H23" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I23" s="44" t="str">
+      <x:c r="I23" s="52" t="str">
         <x:v>Proibir o cadastro sem enviar nenhum nome</x:v>
       </x:c>
-      <x:c r="J23" s="44" t="str">
+      <x:c r="J23" s="52" t="str">
         <x:v>Ao não enviar o campo de nome no cadastro, é esperado que o cadastro seja negado, porém, ele aceita e cadastra a simulação mesmo assim.</x:v>
       </x:c>
-      <x:c r="K23" s="44" t="str">
+      <x:c r="K23" s="52" t="str">
         <x:v>Negar operação quando nome obrigatório estiver vazio ou ausente.</x:v>
       </x:c>
-      <x:c r="L23" s="44" t="str">
+      <x:c r="L23" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M23" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N23" s="44" t="str">
-        <x:v>Bug, POST, Simulações</x:v>
-      </x:c>
-      <x:c r="O23" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="64.5" customHeight="1">
-      <x:c r="A24" s="43" t="str">
+      <x:c r="M23"/>
+      <x:c r="N23"/>
+      <x:c r="O23"/>
+    </x:row>
+    <x:row r="24" ht="84" customHeight="1">
+      <x:c r="A24" s="52" t="str">
         <x:v>BUG-023</x:v>
       </x:c>
-      <x:c r="B24" s="44" t="str">
+      <x:c r="B24" s="52" t="str">
         <x:v>#23</x:v>
       </x:c>
-      <x:c r="C24" s="44" t="str">
+      <x:c r="C24" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D24" s="44" t="str">
+      <x:c r="D24" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E24" s="44" t="str">
+      <x:c r="E24" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F24" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G24" s="44" t="str">
+      <x:c r="F24" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G24" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H24" s="44" t="str">
+      <x:c r="H24" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I24" s="44" t="str">
+      <x:c r="I24" s="52" t="str">
         <x:v>Proibir cadastro de simulação enviando parcela acima de que 48</x:v>
       </x:c>
-      <x:c r="J24" s="44" t="str">
+      <x:c r="J24" s="52" t="str">
         <x:v>Ao enviar um número de parcela acima de 48 vezes, o cadastro é para ser negado, porém ele aceita a requisição e cadastra a simulação.</x:v>
       </x:c>
-      <x:c r="K24" s="44" t="str">
+      <x:c r="K24" s="52" t="str">
         <x:v>Negar cadastro com quantidade de parcelas acima do limite permitido.</x:v>
       </x:c>
-      <x:c r="L24" s="44" t="str">
+      <x:c r="L24" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M24" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N24" s="44" t="str">
-        <x:v>Bug, POST, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O24" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="64.5" customHeight="1">
-      <x:c r="A25" s="43" t="str">
+      <x:c r="M24"/>
+      <x:c r="N24"/>
+      <x:c r="O24"/>
+    </x:row>
+    <x:row r="25" ht="84" customHeight="1">
+      <x:c r="A25" s="52" t="str">
         <x:v>BUG-024</x:v>
       </x:c>
-      <x:c r="B25" s="44" t="str">
+      <x:c r="B25" s="52" t="str">
         <x:v>#24</x:v>
       </x:c>
-      <x:c r="C25" s="44" t="str">
+      <x:c r="C25" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D25" s="44" t="str">
+      <x:c r="D25" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E25" s="44" t="str">
+      <x:c r="E25" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F25" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G25" s="44" t="str">
+      <x:c r="F25" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G25" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H25" s="44" t="str">
+      <x:c r="H25" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I25" s="44" t="str">
+      <x:c r="I25" s="52" t="str">
         <x:v>Proibir cadastro ao enviar no campo valor menos de 1000</x:v>
       </x:c>
-      <x:c r="J25" s="44" t="str">
+      <x:c r="J25" s="52" t="str">
         <x:v>Ao enviar um número de valor abaixo de 1000, o cadastro é para ser negado, porém ele aceita a requisição e cadastra a simulação.</x:v>
       </x:c>
-      <x:c r="K25" s="44" t="str">
+      <x:c r="K25" s="52" t="str">
         <x:v>Negar cadastro com valor abaixo do mínimo permitido.</x:v>
       </x:c>
-      <x:c r="L25" s="44" t="str">
+      <x:c r="L25" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M25" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N25" s="44" t="str">
-        <x:v>Bug, POST, Regra de negócio, Simulações</x:v>
-      </x:c>
-      <x:c r="O25" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="64.5" customHeight="1">
-      <x:c r="A26" s="43" t="str">
+      <x:c r="M25"/>
+      <x:c r="N25"/>
+      <x:c r="O25"/>
+    </x:row>
+    <x:row r="26" ht="84" customHeight="1">
+      <x:c r="A26" s="52" t="str">
         <x:v>BUG-025</x:v>
       </x:c>
-      <x:c r="B26" s="44" t="str">
+      <x:c r="B26" s="52" t="str">
         <x:v>#25</x:v>
       </x:c>
-      <x:c r="C26" s="44" t="str">
+      <x:c r="C26" s="52" t="str">
         <x:v>Melhoria</x:v>
       </x:c>
-      <x:c r="D26" s="44" t="str">
+      <x:c r="D26" s="52" t="str">
         <x:v>Baixa</x:v>
       </x:c>
-      <x:c r="E26" s="44" t="str">
+      <x:c r="E26" s="52" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="F26" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G26" s="44" t="str">
+      <x:c r="F26" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G26" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H26" s="44" t="str">
+      <x:c r="H26" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I26" s="44" t="str">
+      <x:c r="I26" s="52" t="str">
         <x:v>Correção de mensagem de resposta ao enviar seguro vazio</x:v>
       </x:c>
-      <x:c r="J26" s="44" t="str">
+      <x:c r="J26" s="52" t="str">
         <x:v>Ao enviar um corpo de requisição faltando o campo seguro, o ideal seria receber uma mensagem de retorno informando para adicionar o seguro ao corpo de requisição, porém nada é recebido após a requisição.</x:v>
       </x:c>
-      <x:c r="K26" s="44" t="str">
+      <x:c r="K26" s="52" t="str">
         <x:v>Retornar validação adequada quando o campo seguro não for enviado.</x:v>
       </x:c>
-      <x:c r="L26" s="44" t="str">
+      <x:c r="L26" s="52" t="str">
         <x:v>Melhora clareza da resposta e previsibilidade da integração.</x:v>
       </x:c>
-      <x:c r="M26" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N26" s="44" t="str">
-        <x:v>Melhoria, POST, Simulações</x:v>
-      </x:c>
-      <x:c r="O26" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="64.5" customHeight="1">
-      <x:c r="A27" s="43" t="str">
+      <x:c r="M26"/>
+      <x:c r="N26"/>
+      <x:c r="O26"/>
+    </x:row>
+    <x:row r="27" ht="84" customHeight="1">
+      <x:c r="A27" s="52" t="str">
         <x:v>BUG-026</x:v>
       </x:c>
-      <x:c r="B27" s="44" t="str">
+      <x:c r="B27" s="52" t="str">
         <x:v>#26</x:v>
       </x:c>
-      <x:c r="C27" s="44" t="str">
+      <x:c r="C27" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D27" s="44" t="str">
+      <x:c r="D27" s="52" t="str">
         <x:v>Alta</x:v>
       </x:c>
-      <x:c r="E27" s="44" t="str">
+      <x:c r="E27" s="52" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F27" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G27" s="44" t="str">
+      <x:c r="F27" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G27" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H27" s="44" t="str">
+      <x:c r="H27" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I27" s="44" t="str">
+      <x:c r="I27" s="52" t="str">
         <x:v>Correção de status code e tratamento de erro de cadastro sem enviar seguro corretamente</x:v>
       </x:c>
-      <x:c r="J27" s="44" t="str">
+      <x:c r="J27" s="52" t="str">
         <x:v>Ao enviar um corpo de requisição faltando o campo seguro, o ideal seria receber um status code igual as outras requisições que forem deixadas em branco, status code de 400, porém uma de 500 é recebida.</x:v>
       </x:c>
-      <x:c r="K27" s="44" t="str">
+      <x:c r="K27" s="52" t="str">
         <x:v>Retornar validação adequada quando o campo seguro não for enviado.</x:v>
       </x:c>
-      <x:c r="L27" s="44" t="str">
+      <x:c r="L27" s="52" t="str">
         <x:v>Permite criação ou alteração de dados inválidos, afetando consistência e confiabilidade da API.</x:v>
       </x:c>
-      <x:c r="M27" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N27" s="44" t="str">
-        <x:v>Bug, Melhoria, POST, Simulações</x:v>
-      </x:c>
-      <x:c r="O27" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="64.5" customHeight="1">
-      <x:c r="A28" s="43" t="str">
+      <x:c r="M27"/>
+      <x:c r="N27"/>
+      <x:c r="O27"/>
+    </x:row>
+    <x:row r="28" ht="84" customHeight="1">
+      <x:c r="A28" s="52" t="str">
         <x:v>BUG-027</x:v>
       </x:c>
-      <x:c r="B28" s="44" t="str">
+      <x:c r="B28" s="52" t="str">
         <x:v>#27</x:v>
       </x:c>
-      <x:c r="C28" s="44" t="str">
+      <x:c r="C28" s="52" t="str">
         <x:v>Bug</x:v>
       </x:c>
-      <x:c r="D28" s="44" t="str">
+      <x:c r="D28" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E28" s="44" t="str">
+      <x:c r="E28" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F28" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G28" s="44" t="str">
+      <x:c r="F28" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G28" s="52" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="H28" s="44" t="str">
+      <x:c r="H28" s="52" t="str">
         <x:v>Simulações</x:v>
       </x:c>
-      <x:c r="I28" s="44" t="str">
+      <x:c r="I28" s="52" t="str">
         <x:v>Correção de consistência dos IDs cadastrados</x:v>
       </x:c>
-      <x:c r="J28" s="44" t="str">
+      <x:c r="J28" s="52" t="str">
         <x:v>Ao tentar realizar um cadastro utilizando a API e ele falhar, ao tentar realizar um cadastro com sucesso, o ID que deveria seguir a ordem numérica não é seguido e ele pula os números de ID dependendo do número de tentativas (Exemplo: se a próxima simulação a ser cadastrada tiver o ID 10 e falhar no cadastro, quando o cadastro for bem sucedido ele não irá ter o ID 10 e sim o 11, contando a falha como parte dos IDs)</x:v>
       </x:c>
-      <x:c r="K28" s="44" t="str">
+      <x:c r="K28" s="52" t="str">
         <x:v>Manter consistência sequencial dos IDs para cadastros efetivamente concluídos.</x:v>
       </x:c>
-      <x:c r="L28" s="44" t="str">
+      <x:c r="L28" s="52" t="str">
         <x:v>Afeta aderência às regras de negócio e previsibilidade do contrato da API.</x:v>
       </x:c>
-      <x:c r="M28" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N28" s="44" t="str">
-        <x:v>Bug, POST, Simulações</x:v>
-      </x:c>
-      <x:c r="O28" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="64.5" customHeight="1">
-      <x:c r="A29" s="43" t="str">
+      <x:c r="M28"/>
+      <x:c r="N28"/>
+      <x:c r="O28"/>
+    </x:row>
+    <x:row r="29" ht="84" customHeight="1">
+      <x:c r="A29" s="52" t="str">
         <x:v>BUG-028</x:v>
       </x:c>
-      <x:c r="B29" s="44" t="str">
+      <x:c r="B29" s="52" t="str">
         <x:v>#28</x:v>
       </x:c>
-      <x:c r="C29" s="44" t="str">
+      <x:c r="C29" s="52" t="str">
         <x:v>Fluxo</x:v>
       </x:c>
-      <x:c r="D29" s="44" t="str">
+      <x:c r="D29" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E29" s="44" t="str">
+      <x:c r="E29" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F29" s="44" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G29" s="44" t="str">
+      <x:c r="F29" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G29" s="52" t="str">
         <x:v>Fluxo</x:v>
       </x:c>
-      <x:c r="H29" s="44" t="str">
+      <x:c r="H29" s="52" t="str">
         <x:v>Fluxo integrado</x:v>
       </x:c>
-      <x:c r="I29" s="44" t="str">
+      <x:c r="I29" s="52" t="str">
         <x:v>Fluxo de CPF com restrição deve ser interrompido após a verificação de restrições</x:v>
       </x:c>
-      <x:c r="J29" s="44" t="str">
+      <x:c r="J29" s="52" t="str">
         <x:v>Foi realizado um teste de fluxo para verificar se o fluxo de usuário é interrompido após a utilização de um CPF que possui restrição, e como demonstrado, ele funciona corretamente para analisar a restrição, porém o fluxo não é interrompido.</x:v>
       </x:c>
-      <x:c r="K29" s="44" t="str">
+      <x:c r="K29" s="52" t="str">
         <x:v>Aplicar a regra de restrição de CPF e retornar mensagem no padrão documentado.</x:v>
       </x:c>
-      <x:c r="L29" s="44" t="str">
+      <x:c r="L29" s="52" t="str">
         <x:v>Permite continuidade do fluxo mesmo quando uma condição obrigatória deveria bloquear o usuário.</x:v>
       </x:c>
-      <x:c r="M29" s="44" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N29" s="44" t="str">
-        <x:v>Fluxo, Melhoria</x:v>
-      </x:c>
-      <x:c r="O29" s="45" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="64.5" customHeight="1">
-      <x:c r="A30" s="46" t="str">
+      <x:c r="M29"/>
+      <x:c r="N29"/>
+      <x:c r="O29"/>
+    </x:row>
+    <x:row r="30" ht="84" customHeight="1">
+      <x:c r="A30" s="52" t="str">
         <x:v>BUG-029</x:v>
       </x:c>
-      <x:c r="B30" s="47" t="str">
+      <x:c r="B30" s="52" t="str">
         <x:v>#29</x:v>
       </x:c>
-      <x:c r="C30" s="47" t="str">
+      <x:c r="C30" s="52" t="str">
         <x:v>Fluxo</x:v>
       </x:c>
-      <x:c r="D30" s="47" t="str">
+      <x:c r="D30" s="52" t="str">
         <x:v>Média</x:v>
       </x:c>
-      <x:c r="E30" s="47" t="str">
+      <x:c r="E30" s="52" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F30" s="47" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="G30" s="47" t="str">
+      <x:c r="F30" s="52" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="G30" s="52" t="str">
         <x:v>Fluxo</x:v>
       </x:c>
-      <x:c r="H30" s="47" t="str">
+      <x:c r="H30" s="52" t="str">
         <x:v>Fluxo integrado</x:v>
       </x:c>
-      <x:c r="I30" s="47" t="str">
+      <x:c r="I30" s="52" t="str">
         <x:v>Fluxo de CPF vazio deve ser interrompido na verificação de restrições</x:v>
       </x:c>
-      <x:c r="J30" s="47" t="str">
+      <x:c r="J30" s="52" t="str">
         <x:v>Foi realizado um teste de fluxo para verificar se o fluxo de usuário é interrompido após não informar nenhum CPF durante o GET de restrições, e como demonstrado, ele não demonstra nenhuma informação que o CPF está vazio durante todo o fluxo de usuário e o fluxo não é interrompido.</x:v>
       </x:c>
-      <x:c r="K30" s="47" t="str">
+      <x:c r="K30" s="52" t="str">
         <x:v>Negar operação quando CPF obrigatório estiver vazio ou ausente.</x:v>
       </x:c>
-      <x:c r="L30" s="47" t="str">
+      <x:c r="L30" s="52" t="str">
         <x:v>Permite continuidade do fluxo mesmo quando uma condição obrigatória deveria bloquear o usuário.</x:v>
       </x:c>
-      <x:c r="M30" s="47" t="str">
-        <x:v>Evidência anexada no registro original do projeto</x:v>
-      </x:c>
-      <x:c r="N30" s="47" t="str">
-        <x:v>Fluxo, Melhoria</x:v>
-      </x:c>
-      <x:c r="O30" s="48" t="str">
-        <x:v>17/05/2024</x:v>
-      </x:c>
+      <x:c r="M30"/>
+      <x:c r="N30"/>
+      <x:c r="O30"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="D2:D30">
@@ -2553,7 +2399,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dbd8768b5604ea5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ea62792220d4aae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2704,6 +2550,6 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8052e5c28a70485f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R067a46a376644bd2"/>
 </x:worksheet>
 </file>
</xml_diff>